<commit_message>
[FIX] xlsx: handle composite ranges in chart data conversion
In Excel, we can write range union `(A1:A3,A1:C3)` and range
intersections `(A1:A3 A1:C3)`. We do not support them at the moment,
having them in a chart datasets/labels would crash. We will drop those
ranges in the chart data conversion.

As far as I can tell, the only other place we can use those types of
ranges is in formulas/Named Ranges. We can leave those, as they will simply
fail the parsing and produce #BAD_EXPR/#REF.

closes odoo/o-spreadsheet#9913

Task: 5503375
X-original-commit: 672495811b499193cd4c2e3ba0ef519c0efb32a7
Signed-off-by: Rémi Rahir (rar) <rar@odoo.com>
Signed-off-by: Adrien Minne (adrm) <adrm@odoo.com>
</commit_message>
<xml_diff>
--- a/tests/__xlsx__/xlsx_demo_data.xlsx
+++ b/tests/__xlsx__/xlsx_demo_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Odoo\spreadsheet\tests\__xlsx__\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\odoo\spreadsheet\tests\__xlsx__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F832354-F3E9-4BC5-A260-88E8A391D52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D70715-801F-423D-A719-873B16295B9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,10 +30,11 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId15"/>
+    <externalReference r:id="rId16"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId16"/>
+    <pivotCache cacheId="1" r:id="rId17"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -2151,7 +2152,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2335,6 +2336,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2351,21 +2365,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -2812,7 +2811,7 @@
         <u/>
         <color theme="7"/>
       </font>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="170" formatCode="dd/mm/yyyy"/>
       <fill>
         <patternFill patternType="lightTrellis">
           <fgColor theme="4"/>
@@ -3958,6 +3957,514 @@
 </file>
 
 <file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr b="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="2200"/>
+              <a:t>chart with composite ranges</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7030A0"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="7030A0"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>([2]Sheet1!$A$27:$C$35,[2]Sheet1!$A$27:$C$31)</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="14"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>24</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>12</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>27</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>9</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>45</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>17</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>43</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>11</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>16</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>24</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>12</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>27</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>9</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>45</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>12</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>48</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>45</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>1</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>25</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>31</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>20</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>19</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>16</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>12</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>48</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>45</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>1</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>25</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Emily Anderson (Emmy)</c:v>
+                  </c:pt>
+                  <c:pt idx="1">
+                    <c:v>Sophie Allen (Saffi)</c:v>
+                  </c:pt>
+                  <c:pt idx="2">
+                    <c:v>Chloe Adams</c:v>
+                  </c:pt>
+                  <c:pt idx="3">
+                    <c:v>Megan Alexander (Meg)</c:v>
+                  </c:pt>
+                  <c:pt idx="4">
+                    <c:v>Lucy Arnold (Lulu)</c:v>
+                  </c:pt>
+                  <c:pt idx="5">
+                    <c:v>Hannah Alvarez</c:v>
+                  </c:pt>
+                  <c:pt idx="6">
+                    <c:v>Jessica Alcock (Jess)</c:v>
+                  </c:pt>
+                  <c:pt idx="7">
+                    <c:v>Charlotte Anaya</c:v>
+                  </c:pt>
+                  <c:pt idx="8">
+                    <c:v>Lauren Anthony</c:v>
+                  </c:pt>
+                  <c:pt idx="9">
+                    <c:v>Emily Anderson (Emmy)</c:v>
+                  </c:pt>
+                  <c:pt idx="10">
+                    <c:v>Sophie Allen (Saffi)</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>Chloe Adams</c:v>
+                  </c:pt>
+                  <c:pt idx="12">
+                    <c:v>Megan Alexander (Meg)</c:v>
+                  </c:pt>
+                  <c:pt idx="13">
+                    <c:v>Lucy Arnold (Lulu)</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[2]Sheet1!$B$27:$B$31</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:solidFill>
+                      <a:srgbClr val="7030A0"/>
+                    </a:solidFill>
+                    <a:prstDash val="solid"/>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A1E9-46C7-8442-4AB5744608FB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C65911"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="C65911"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="1"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>[2]Sheet1!$A$27:$A$31</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Emily Anderson (Emmy)</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sophie Allen (Saffi)</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Chloe Adams</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Megan Alexander (Meg)</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Lucy Arnold (Lulu)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[2]Sheet1!$C$27:$C$31</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>45</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
+              <c14:invertSolidFillFmt>
+                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                  <a:ln>
+                    <a:solidFill>
+                      <a:srgbClr val="C65911"/>
+                    </a:solidFill>
+                    <a:prstDash val="solid"/>
+                  </a:ln>
+                </c14:spPr>
+              </c14:invertSolidFillFmt>
+            </c:ext>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A1E9-46C7-8442-4AB5744608FB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="70"/>
+        <c:overlap val="-20"/>
+        <c:axId val="17781237"/>
+        <c:axId val="88853993"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="17781237"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="1"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr sz="1000" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="88853993"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="1"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="88853993"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="B7B7B7"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr lvl="0">
+                  <a:defRPr b="0">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="1"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr lvl="0">
+              <a:defRPr sz="1000" b="0" i="0">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="17781237"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr lvl="0">
+            <a:defRPr sz="1000" b="0" i="0">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="fr-FR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="zero"/>
+    <c:showDLblsOverMax val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln cmpd="sng">
+      <a:solidFill>
+        <a:srgbClr val="000000"/>
+      </a:solidFill>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -8578,6 +9085,47 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="12" name="Chart 11" title="Chart">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F47B043-E8D8-482A-8380-D03C8E238CC3}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{00000000-0008-0000-0100-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -8702,6 +9250,9 @@
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:relativeUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Feuil1"/>
     </sheetNames>
@@ -8713,6 +9264,149 @@
           </cell>
         </row>
       </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+      <sheetName val="Formulas"/>
+      <sheetName val="jestSheet"/>
+      <sheetName val="jestStyles"/>
+      <sheetName val="jestCfs"/>
+      <sheetName val="jestTable"/>
+      <sheetName val="jestPivot"/>
+      <sheetName val="jestCharts"/>
+      <sheetName val="jestMiscTest"/>
+      <sheetName val="jestHiddenSheet"/>
+      <sheetName val="jestFreezePane"/>
+      <sheetName val="jestImages"/>
+      <sheetName val="jestOneCellAnchor"/>
+      <sheetName val="jestDataValidations"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="27">
+          <cell r="A27" t="str">
+            <v>Emily Anderson (Emmy)</v>
+          </cell>
+          <cell r="B27">
+            <v>12</v>
+          </cell>
+          <cell r="C27">
+            <v>24</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="A28" t="str">
+            <v>Sophie Allen (Saffi)</v>
+          </cell>
+          <cell r="B28">
+            <v>48</v>
+          </cell>
+          <cell r="C28">
+            <v>12</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="A29" t="str">
+            <v>Chloe Adams</v>
+          </cell>
+          <cell r="B29">
+            <v>45</v>
+          </cell>
+          <cell r="C29">
+            <v>27</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="A30" t="str">
+            <v>Megan Alexander (Meg)</v>
+          </cell>
+          <cell r="B30">
+            <v>1</v>
+          </cell>
+          <cell r="C30">
+            <v>9</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="A31" t="str">
+            <v>Lucy Arnold (Lulu)</v>
+          </cell>
+          <cell r="B31">
+            <v>25</v>
+          </cell>
+          <cell r="C31">
+            <v>45</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="A32" t="str">
+            <v>Hannah Alvarez</v>
+          </cell>
+          <cell r="B32">
+            <v>31</v>
+          </cell>
+          <cell r="C32">
+            <v>17</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="A33" t="str">
+            <v>Jessica Alcock (Jess)</v>
+          </cell>
+          <cell r="B33">
+            <v>20</v>
+          </cell>
+          <cell r="C33">
+            <v>43</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="A34" t="str">
+            <v>Charlotte Anaya</v>
+          </cell>
+          <cell r="B34">
+            <v>19</v>
+          </cell>
+          <cell r="C34">
+            <v>11</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="A35" t="str">
+            <v>Lauren Anthony</v>
+          </cell>
+          <cell r="B35">
+            <v>16</v>
+          </cell>
+          <cell r="C35">
+            <v>16</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -8837,7 +9531,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9B3CE3F5-58D8-48A3-B9C6-24D1506C9F5C}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="C3:L21" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -9463,10 +10157,10 @@
       <c r="G2" s="104">
         <v>5</v>
       </c>
-      <c r="H2" s="105" t="s">
+      <c r="H2" s="110" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="106"/>
+      <c r="I2" s="111"/>
       <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9476,10 +10170,10 @@
       <c r="G3" s="104">
         <v>8</v>
       </c>
-      <c r="H3" s="106"/>
-      <c r="I3" s="106"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="107">
+      <c r="K3" s="112">
         <v>5</v>
       </c>
       <c r="L3" s="6"/>
@@ -9497,10 +10191,10 @@
       <c r="G4" s="104">
         <v>9</v>
       </c>
-      <c r="H4" s="106"/>
-      <c r="I4" s="106"/>
+      <c r="H4" s="111"/>
+      <c r="I4" s="111"/>
       <c r="J4" s="5"/>
-      <c r="K4" s="108"/>
+      <c r="K4" s="113"/>
       <c r="L4" s="6"/>
     </row>
     <row r="5" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9510,10 +10204,10 @@
       <c r="G5" s="104">
         <v>15</v>
       </c>
-      <c r="H5" s="106"/>
-      <c r="I5" s="106"/>
+      <c r="H5" s="111"/>
+      <c r="I5" s="111"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="108"/>
+      <c r="K5" s="113"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9521,7 +10215,7 @@
         <v>22</v>
       </c>
       <c r="J6" s="5"/>
-      <c r="K6" s="108"/>
+      <c r="K6" s="113"/>
       <c r="L6" s="6"/>
     </row>
     <row r="7" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9529,7 +10223,7 @@
         <v>3</v>
       </c>
       <c r="J7" s="5"/>
-      <c r="K7" s="108"/>
+      <c r="K7" s="113"/>
       <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9537,7 +10231,7 @@
         <v>30</v>
       </c>
       <c r="J8" s="5"/>
-      <c r="K8" s="109"/>
+      <c r="K8" s="114"/>
       <c r="L8" s="6"/>
     </row>
     <row r="9" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -9936,63 +10630,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="106" t="s">
         <v>423</v>
       </c>
-      <c r="B1" s="113" t="s">
+      <c r="B1" s="107" t="s">
         <v>424</v>
       </c>
-      <c r="C1" s="113" t="s">
+      <c r="C1" s="107" t="s">
         <v>425</v>
       </c>
-      <c r="D1" s="113" t="s">
+      <c r="D1" s="107" t="s">
         <v>426</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="E1" s="107" t="s">
         <v>427</v>
       </c>
-      <c r="F1" s="113" t="s">
+      <c r="F1" s="107" t="s">
         <v>428</v>
       </c>
-      <c r="G1" s="113" t="s">
+      <c r="G1" s="107" t="s">
         <v>429</v>
       </c>
-      <c r="H1" s="113" t="s">
+      <c r="H1" s="107" t="s">
         <v>430</v>
       </c>
-      <c r="I1" s="114" t="s">
+      <c r="I1" s="108" t="s">
         <v>431</v>
       </c>
-      <c r="J1" s="111" t="s">
+      <c r="J1" s="105" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="115">
+      <c r="A2">
         <v>4</v>
       </c>
-      <c r="B2" s="115">
+      <c r="B2">
         <v>99.5</v>
       </c>
-      <c r="C2" s="115">
-        <v>1</v>
-      </c>
-      <c r="D2" s="115" t="s">
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>432</v>
       </c>
-      <c r="E2" s="116">
+      <c r="E2" s="39">
         <v>45575</v>
       </c>
-      <c r="F2" s="117">
+      <c r="F2" s="109">
         <v>0.64583333333333337</v>
       </c>
-      <c r="G2" s="117" t="s">
+      <c r="G2" s="109" t="s">
         <v>433</v>
       </c>
-      <c r="H2" s="116">
+      <c r="H2" s="39">
         <v>45292</v>
       </c>
-      <c r="I2" s="115">
+      <c r="I2">
         <v>4</v>
       </c>
       <c r="J2">
@@ -10000,31 +10694,31 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="115">
+      <c r="A3">
         <v>3</v>
       </c>
-      <c r="B3" s="115">
+      <c r="B3">
         <v>40</v>
       </c>
-      <c r="C3" s="115">
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="115" t="s">
+      <c r="D3" t="s">
         <v>434</v>
       </c>
-      <c r="E3" s="116">
+      <c r="E3" s="39">
         <v>45576</v>
       </c>
-      <c r="F3" s="117">
+      <c r="F3" s="109">
         <v>0.57638888888888884</v>
       </c>
-      <c r="G3" s="117" t="s">
+      <c r="G3" s="109" t="s">
         <v>435</v>
       </c>
-      <c r="H3" s="116">
+      <c r="H3" s="39">
         <v>45231</v>
       </c>
-      <c r="I3" s="115" t="s">
+      <c r="I3" t="s">
         <v>433</v>
       </c>
       <c r="J3">
@@ -10032,31 +10726,31 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="115">
+      <c r="A4">
         <v>9</v>
       </c>
-      <c r="B4" s="115">
+      <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4" s="115">
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="D4" s="115" t="s">
+      <c r="D4" t="s">
         <v>436</v>
       </c>
-      <c r="E4" s="116">
+      <c r="E4" s="39">
         <v>45574</v>
       </c>
-      <c r="F4" s="117">
+      <c r="F4" s="109">
         <v>0.73958333333333337</v>
       </c>
-      <c r="G4" s="117" t="s">
+      <c r="G4" s="109" t="s">
         <v>437</v>
       </c>
-      <c r="H4" s="116">
+      <c r="H4" s="39">
         <v>45325</v>
       </c>
-      <c r="I4" s="115">
+      <c r="I4">
         <v>3</v>
       </c>
       <c r="J4">
@@ -10064,31 +10758,31 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="115">
+      <c r="A5">
         <v>5</v>
       </c>
-      <c r="B5" s="115">
+      <c r="B5">
         <v>120</v>
       </c>
-      <c r="C5" s="115">
+      <c r="C5">
         <v>4</v>
       </c>
-      <c r="D5" s="115" t="s">
+      <c r="D5" t="s">
         <v>434</v>
       </c>
-      <c r="E5" s="116">
+      <c r="E5" s="39">
         <v>45573</v>
       </c>
-      <c r="F5" s="117">
+      <c r="F5" s="109">
         <v>0.66666666666666663</v>
       </c>
-      <c r="G5" s="115" t="s">
+      <c r="G5" t="s">
         <v>438</v>
       </c>
-      <c r="H5" s="116">
+      <c r="H5" s="39">
         <v>45084</v>
       </c>
-      <c r="I5" s="115">
+      <c r="I5">
         <v>3</v>
       </c>
       <c r="J5">
@@ -10096,31 +10790,31 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="115">
+      <c r="A6">
         <v>7</v>
       </c>
-      <c r="B6" s="115">
+      <c r="B6">
         <v>12</v>
       </c>
-      <c r="C6" s="115">
+      <c r="C6">
         <v>5</v>
       </c>
-      <c r="D6" s="115" t="s">
+      <c r="D6" t="s">
         <v>436</v>
       </c>
-      <c r="E6" s="116">
+      <c r="E6" s="39">
         <v>45566</v>
       </c>
-      <c r="F6" s="117">
+      <c r="F6" s="109">
         <v>0.5229166666666667</v>
       </c>
-      <c r="G6" s="115" t="s">
+      <c r="G6" t="s">
         <v>439</v>
       </c>
-      <c r="H6" s="116">
+      <c r="H6" s="39">
         <v>45420</v>
       </c>
-      <c r="I6" s="115" t="s">
+      <c r="I6" t="s">
         <v>438</v>
       </c>
       <c r="J6">
@@ -12028,7 +12722,7 @@
       </c>
       <c r="B100" s="19">
         <f ca="1">NOW()</f>
-        <v>45938.493500231481</v>
+        <v>46316.424889236114</v>
       </c>
       <c r="D100" s="104">
         <f ca="1">IF(ISNUMBER(B100),1,0)</f>
@@ -12718,7 +13412,7 @@
       </c>
       <c r="B144" s="18">
         <f ca="1">TODAY()</f>
-        <v>45938</v>
+        <v>46316</v>
       </c>
       <c r="D144" s="104">
         <f ca="1">IF(ISNUMBER(B144),1,0)</f>
@@ -13067,10 +13761,10 @@
       <c r="C1" t="s">
         <v>231</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="115" t="s">
         <v>232</v>
       </c>
-      <c r="E1" s="110"/>
+      <c r="E1" s="115"/>
       <c r="F1" t="s">
         <v>233</v>
       </c>
@@ -13083,8 +13777,8 @@
         <f>SUM(A1)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="110"/>
-      <c r="E2" s="110"/>
+      <c r="D2" s="115"/>
+      <c r="E2" s="115"/>
       <c r="H2" t="str">
         <f>[1]Feuil1!$A$1</f>
         <v>referenced string</v>
@@ -13120,21 +13814,21 @@
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" cm="1">
         <f t="array" aca="1" ref="A30:B31" ca="1">_xlfn.RANDARRAY(2,2)</f>
-        <v>0.7272925709748963</v>
+        <v>0.78768916454204807</v>
       </c>
       <c r="B30">
         <f ca="1"/>
-        <v>0.95782684877879687</v>
+        <v>0.98576428000403649</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <f ca="1"/>
-        <v>0.31704384406036645</v>
+        <v>0.3036437649516297</v>
       </c>
       <c r="B31">
         <f ca="1"/>
-        <v>8.7112099778747121E-2</v>
+        <v>9.0519996913986489E-2</v>
       </c>
     </row>
   </sheetData>
@@ -13768,7 +14462,7 @@
       </c>
       <c r="B12" s="39">
         <f ca="1">TODAY()</f>
-        <v>45938</v>
+        <v>46316</v>
       </c>
       <c r="C12" s="39">
         <f>DATE(2010,10,2)</f>

</xml_diff>